<commit_message>
Fixed typos in Recommendations
</commit_message>
<xml_diff>
--- a/week-01/Kuppi Coffee Company Customer Satisfaction Survey.xlsx
+++ b/week-01/Kuppi Coffee Company Customer Satisfaction Survey.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sguer\Documents\DataAnalytics\week-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{931F7FDD-EB51-4634-B900-B1B2C4069461}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92FEB60B-6B5F-4C98-9442-D5FA6DC64DA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5115" yWindow="525" windowWidth="16485" windowHeight="12060" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5115" yWindow="525" windowWidth="16485" windowHeight="12060" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Survey_Responses" sheetId="1" r:id="rId1"/>
@@ -384,18 +384,6 @@
   </cellStyles>
   <dxfs count="42">
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="28" formatCode="mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
-    </dxf>
-    <dxf>
       <border>
         <left style="thin">
           <color indexed="64"/>
@@ -681,6 +669,9 @@
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="0" formatCode="General"/>
       <alignment horizontal="general" vertical="center" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -702,11 +693,20 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="28" formatCode="mm:ss"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="28" formatCode="mm:ss"/>
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
       <alignment vertical="center" textRotation="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="164" formatCode="mm/dd/yyyy\ hh:mm:ss"/>
@@ -5338,7 +5338,7 @@
       <xdr:row>0</xdr:row>
       <xdr:rowOff>128586</xdr:rowOff>
     </xdr:from>
-    <xdr:ext cx="5276850" cy="3192412"/>
+    <xdr:ext cx="5276850" cy="3536866"/>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
         <xdr:cNvPr id="2" name="TextBox 1">
@@ -5353,7 +5353,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="214313" y="128586"/>
-          <a:ext cx="5276850" cy="3192412"/>
+          <a:ext cx="5276850" cy="3536866"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -5382,41 +5382,90 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
+          <a:pPr rtl="0"/>
           <a:r>
-            <a:rPr lang="en-US" sz="1100"/>
-            <a:t>Survey</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t> results indicate that although Kuppi Coffee Company has a relatively new consumer base, the overall customer satisfaction rate is a five out of five, largely due to the in-store experience and anemities, which collective has an average rating of 4.6</a:t>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Survey results indicate that although Kuppi Coffee Company has a relatively new consumer base, the overall customer satisfaction rate is a five out of five, largely due to the in-store experience and amenities, which collective has an average rating of 4.6</a:t>
           </a:r>
         </a:p>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
+          <a:pPr rtl="0"/>
+          <a:endParaRPr lang="en-US" b="0">
+            <a:effectLst/>
+          </a:endParaRPr>
         </a:p>
         <a:p>
+          <a:pPr rtl="0"/>
           <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t>Additonally, survey responses indicate that 60% of respondents said yes to a loyalty rewards program, with the remaining 40% expressiong conditional interest depending on the rewards offered. Overall, no respondents were opposed to the program, with 80% preferring a points-based system over a punch-card style loyalty program.</a:t>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Additionally, survey responses indicate that 60% of respondents said yes to a loyalty rewards program, with the remaining 40% expressing conditional interest depending on the rewards offered. Overall, no respondents were opposed to the program, with 80% preferring a points-based system over a punch-card style loyalty program.</a:t>
           </a:r>
         </a:p>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
+          <a:pPr rtl="0"/>
+          <a:endParaRPr lang="en-US" b="0">
+            <a:effectLst/>
+          </a:endParaRPr>
         </a:p>
         <a:p>
+          <a:pPr rtl="0"/>
           <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t>Results indicate that the top preferred reward is a points-based redemption system where customers earn one point for every dollar spent, with the opprotuntiy to redeem points for free specialty drinks or food items. This aligns with pruchase trends, as specialty coffee drinks and breakfast sandwiches are the most frequently ordered items.</a:t>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>Results indicate that the top preferred reward is a points-based redemption system where customers earn one point for every dollar spent, with the opportunity to redeem points for free specialty drinks or food items. This aligns with purchase trends, as specialty coffee drinks and breakfast sandwiches are the most frequently ordered items.</a:t>
           </a:r>
         </a:p>
         <a:p>
-          <a:endParaRPr lang="en-US" sz="1100" baseline="0"/>
+          <a:pPr rtl="0"/>
+          <a:endParaRPr lang="en-US" b="0">
+            <a:effectLst/>
+          </a:endParaRPr>
         </a:p>
         <a:p>
+          <a:pPr rtl="0"/>
           <a:r>
-            <a:rPr lang="en-US" sz="1100" baseline="0"/>
-            <a:t>To expand Kuppi's clientele and convert its new cosumer base into loyal customers, a points-based redeemtion loyalty program that targets specialtiy drinks and food purchases would likely yield the best resutls, as long as food and beveagre quality and the in-store expeirence remain high. </a:t>
+            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+              <a:effectLst/>
+              <a:latin typeface="+mn-lt"/>
+              <a:ea typeface="+mn-ea"/>
+              <a:cs typeface="+mn-cs"/>
+            </a:rPr>
+            <a:t>To expand Kuppi's clientele and convert its new consumer base into loyal customers, a points-based redemption loyalty program that targets specialty drinks and food purchases would likely yield the best results, as long as food and beverage quality and the in-store experience remain high. </a:t>
           </a:r>
+          <a:endParaRPr lang="en-US" b="0">
+            <a:effectLst/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
+          <a:br>
+            <a:rPr lang="en-US"/>
+          </a:br>
           <a:endParaRPr lang="en-US" sz="1100"/>
         </a:p>
       </xdr:txBody>
@@ -5689,35 +5738,35 @@
     <dataField name="Count of System" fld="17" subtotal="count" baseField="16" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="12">
+    <format dxfId="8">
       <pivotArea dataOnly="0" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="11">
+    <format dxfId="7">
       <pivotArea dataOnly="0" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="10">
+    <format dxfId="6">
       <pivotArea field="16" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="9">
+    <format dxfId="5">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="8">
+    <format dxfId="4">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="7">
+    <format dxfId="3">
       <pivotArea field="16" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="6">
+    <format dxfId="2">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="16" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="5">
+    <format dxfId="1">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="4">
+    <format dxfId="0">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -5822,13 +5871,13 @@
     <dataField name="Count of Interest" fld="0" subtotal="count" baseField="15" baseItem="0"/>
   </dataFields>
   <formats count="9">
-    <format dxfId="21">
+    <format dxfId="17">
       <pivotArea field="15" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="20">
+    <format dxfId="16">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
-    <format dxfId="19">
+    <format dxfId="15">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="15" count="1">
@@ -5837,26 +5886,26 @@
         </references>
       </pivotArea>
     </format>
-    <format dxfId="18">
+    <format dxfId="14">
       <pivotArea type="all" dataOnly="0" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="17">
+    <format dxfId="13">
       <pivotArea outline="0" collapsedLevelsAreSubtotals="1" fieldPosition="0"/>
     </format>
-    <format dxfId="16">
+    <format dxfId="12">
       <pivotArea field="15" type="button" dataOnly="0" labelOnly="1" outline="0" axis="axisRow" fieldPosition="0"/>
     </format>
-    <format dxfId="15">
+    <format dxfId="11">
       <pivotArea dataOnly="0" labelOnly="1" fieldPosition="0">
         <references count="1">
           <reference field="15" count="0"/>
         </references>
       </pivotArea>
     </format>
-    <format dxfId="14">
+    <format dxfId="10">
       <pivotArea dataOnly="0" labelOnly="1" grandRow="1" outline="0" fieldPosition="0"/>
     </format>
-    <format dxfId="13">
+    <format dxfId="9">
       <pivotArea dataOnly="0" labelOnly="1" outline="0" axis="axisValues" fieldPosition="0"/>
     </format>
   </formats>
@@ -5897,43 +5946,43 @@
   <autoFilter ref="A1:S6" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
   <tableColumns count="19">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="ID" dataDxfId="40"/>
-    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Start time" dataDxfId="39" totalsRowDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Completion time" dataDxfId="38" totalsRowDxfId="2"/>
-    <tableColumn id="21" xr3:uid="{574F5E68-45C2-4C0B-B4DD-7D02BE97E8A1}" name="Time to Complete" totalsRowFunction="custom" dataDxfId="37" totalsRowDxfId="1">
+    <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Start time" dataDxfId="39" totalsRowDxfId="38"/>
+    <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Completion time" dataDxfId="37" totalsRowDxfId="36"/>
+    <tableColumn id="21" xr3:uid="{574F5E68-45C2-4C0B-B4DD-7D02BE97E8A1}" name="Time to Complete" totalsRowFunction="custom" dataDxfId="35" totalsRowDxfId="34">
       <calculatedColumnFormula>C2-B2</calculatedColumnFormula>
       <totalsRowFormula>AVERAGE(D2:D6)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="36"/>
-    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="How often do you visit Kuppi Coffee?" dataDxfId="35"/>
-    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="How satisfied are you with your overall experience at our cafe? (1 = Very Dissatisfied → 5 = Very Satisfied)" totalsRowFunction="custom" dataDxfId="34">
+    <tableColumn id="4" xr3:uid="{00000000-0010-0000-0000-000004000000}" name="Email" dataDxfId="33"/>
+    <tableColumn id="7" xr3:uid="{00000000-0010-0000-0000-000007000000}" name="How often do you visit Kuppi Coffee?" dataDxfId="32"/>
+    <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="How satisfied are you with your overall experience at our cafe? (1 = Very Dissatisfied → 5 = Very Satisfied)" totalsRowFunction="custom" dataDxfId="31">
       <totalsRowFormula>AVERAGE(G2:G6)</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Which of the following do you typically order at Kuppi Coffee? (select all that apply)" dataDxfId="33"/>
-    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Staff Friendliness" totalsRowFunction="custom" dataDxfId="32" totalsRowDxfId="0">
+    <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="Which of the following do you typically order at Kuppi Coffee? (select all that apply)" dataDxfId="30"/>
+    <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="Staff Friendliness" totalsRowFunction="custom" dataDxfId="29" totalsRowDxfId="28">
       <totalsRowFormula array="1">AVERAGE(_xlfn.SWITCH(I2:I6,"Very Dissatisfied",1,"Dissatisfied",2,"Neutral",3,"Satisfied",4,"Very Satisfied",5))</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Speed of Service" totalsRowFunction="custom" dataDxfId="31">
+    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Speed of Service" totalsRowFunction="custom" dataDxfId="27">
       <totalsRowFormula array="1">AVERAGE(_xlfn.SWITCH(J2:J6,"Very Dissatisfied",1,"Dissatisfied",2,"Neutral",3,"Satisfied",4,"Very Satisfied",5))</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Cleanliness" totalsRowFunction="custom" dataDxfId="30">
+    <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="Cleanliness" totalsRowFunction="custom" dataDxfId="26">
       <totalsRowFormula array="1">AVERAGE(_xlfn.SWITCH(K2:K6,"Very Dissatisfied",1,"Dissatisfied",2,"Neutral",3,"Satisfied",4,"Very Satisfied",5))</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Wi-Fi Quality" totalsRowFunction="custom" dataDxfId="29">
+    <tableColumn id="13" xr3:uid="{00000000-0010-0000-0000-00000D000000}" name="Wi-Fi Quality" totalsRowFunction="custom" dataDxfId="25">
       <totalsRowFormula array="1">AVERAGE(_xlfn.SWITCH(L2:L6,"Very Dissatisfied",1,"Dissatisfied",2,"Neutral",3,"Satisfied",4,"Very Satisfied",5))</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Seating Comfort" totalsRowFunction="custom" dataDxfId="28">
+    <tableColumn id="14" xr3:uid="{00000000-0010-0000-0000-00000E000000}" name="Seating Comfort" totalsRowFunction="custom" dataDxfId="24">
       <totalsRowFormula array="1">AVERAGE(_xlfn.SWITCH(M2:M6,"Very Dissatisfied",1,"Dissatisfied",2,"Neutral",3,"Satisfied",4,"Very Satisfied",5))</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Food &amp; Drink Quality" totalsRowFunction="custom" dataDxfId="27">
+    <tableColumn id="15" xr3:uid="{00000000-0010-0000-0000-00000F000000}" name="Food &amp; Drink Quality" totalsRowFunction="custom" dataDxfId="23">
       <totalsRowFormula array="1">AVERAGE(_xlfn.SWITCH(N2:N6,"Very Dissatisfied",1,"Dissatisfied",2,"Neutral",3,"Satisfied",4,"Very Satisfied",5))</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="How likely are you to recommend Kuppi Coffee to someone? (1 = Not at all likely → 10 = Extremely likely)" dataDxfId="26"/>
-    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Would you be interested in a loyalty/rewards program at Kuppi Coffee?" totalsRowFunction="custom" dataDxfId="25">
+    <tableColumn id="16" xr3:uid="{00000000-0010-0000-0000-000010000000}" name="How likely are you to recommend Kuppi Coffee to someone? (1 = Not at all likely → 10 = Extremely likely)" dataDxfId="22"/>
+    <tableColumn id="17" xr3:uid="{00000000-0010-0000-0000-000011000000}" name="Would you be interested in a loyalty/rewards program at Kuppi Coffee?" totalsRowFunction="custom" dataDxfId="21">
       <totalsRowFormula>COUNTIF(P2:P6, "Maybe, depending on the rewards")</totalsRowFormula>
     </tableColumn>
-    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Would you prefer a punch-card style reward or a points-based system? (Please select one)" dataDxfId="24"/>
-    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Please rank the following rewards you would be most interested in (1 = most interest)" dataDxfId="23"/>
-    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Any additional comments or concerns?" dataDxfId="22"/>
+    <tableColumn id="18" xr3:uid="{00000000-0010-0000-0000-000012000000}" name="Would you prefer a punch-card style reward or a points-based system? (Please select one)" dataDxfId="20"/>
+    <tableColumn id="19" xr3:uid="{00000000-0010-0000-0000-000013000000}" name="Please rank the following rewards you would be most interested in (1 = most interest)" dataDxfId="19"/>
+    <tableColumn id="20" xr3:uid="{00000000-0010-0000-0000-000014000000}" name="Any additional comments or concerns?" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium13" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>

</xml_diff>

<commit_message>
Update Kuppi Coffee Survey Results
</commit_message>
<xml_diff>
--- a/week-01/Kuppi Coffee Company Customer Satisfaction Survey.xlsx
+++ b/week-01/Kuppi Coffee Company Customer Satisfaction Survey.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sguer\Documents\DataAnalytics\week-01\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{92FEB60B-6B5F-4C98-9442-D5FA6DC64DA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D715802-FD2B-4F9F-AD7B-E1EBC7A83B69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5115" yWindow="525" windowWidth="16485" windowHeight="12060" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1208" yWindow="442" windowWidth="20025" windowHeight="12061" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Survey_Responses" sheetId="1" r:id="rId1"/>
@@ -5382,30 +5382,28 @@
         </a:bodyPr>
         <a:lstStyle/>
         <a:p>
-          <a:pPr rtl="0"/>
           <a:r>
-            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
+            <a:rPr lang="en-US">
               <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Survey results indicate that although Kuppi Coffee Company has a relatively new consumer base, the overall customer satisfaction rate is a five out of five, largely due to the in-store experience and amenities, which collective has an average rating of 4.6</a:t>
+            <a:t>Survey results indicate that although Kuppi Coffee Company has a relatively new consumer base, the overall customer satisfaction rate is a five out of five, largely due to the in-store experience and amenities,</a:t>
+          </a:r>
+          <a:r>
+            <a:rPr lang="en-US" baseline="0">
+              <a:effectLst/>
+            </a:rPr>
+            <a:t> which collectively has an average rating of 4.6</a:t>
           </a:r>
         </a:p>
         <a:p>
-          <a:pPr rtl="0"/>
-          <a:endParaRPr lang="en-US" b="0">
+          <a:endParaRPr lang="en-US">
             <a:effectLst/>
           </a:endParaRPr>
         </a:p>
         <a:p>
           <a:pPr rtl="0"/>
           <a:r>
-            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:rPr lang="en-US" sz="1100" b="0" i="0">
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
@@ -5416,27 +5414,31 @@
             </a:rPr>
             <a:t>Additionally, survey responses indicate that 60% of respondents said yes to a loyalty rewards program, with the remaining 40% expressing conditional interest depending on the rewards offered. Overall, no respondents were opposed to the program, with 80% preferring a points-based system over a punch-card style loyalty program.</a:t>
           </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr rtl="0"/>
-          <a:endParaRPr lang="en-US" b="0">
+          <a:endParaRPr lang="en-US">
             <a:effectLst/>
           </a:endParaRPr>
         </a:p>
         <a:p>
-          <a:pPr rtl="0"/>
+          <a:endParaRPr lang="en-US">
+            <a:effectLst/>
+          </a:endParaRPr>
+        </a:p>
+        <a:p>
           <a:r>
-            <a:rPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
+            <a:rPr lang="en-US">
               <a:effectLst/>
-              <a:latin typeface="+mn-lt"/>
-              <a:ea typeface="+mn-ea"/>
-              <a:cs typeface="+mn-cs"/>
             </a:rPr>
-            <a:t>Results indicate that the top preferred reward is a points-based redemption system where customers earn one point for every dollar spent, with the opportunity to redeem points for free specialty drinks or food items. This aligns with purchase trends, as specialty coffee drinks and breakfast sandwiches are the most frequently ordered items.</a:t>
+            <a:t>Results indicate that the top preferred reward is a points-based redemption system where customers earn one point for every dollar spent, redeemable for free specialty drinks or food items. This aligns with purchase trends, as specialty coffee drinks and breakfast sandwiches are the most frequently ordered items.</a:t>
           </a:r>
+          <a:endParaRPr lang="en-US" sz="1100" b="0" i="0" u="none" strike="noStrike">
+            <a:solidFill>
+              <a:schemeClr val="tx1"/>
+            </a:solidFill>
+            <a:effectLst/>
+            <a:latin typeface="+mn-lt"/>
+            <a:ea typeface="+mn-ea"/>
+            <a:cs typeface="+mn-cs"/>
+          </a:endParaRPr>
         </a:p>
         <a:p>
           <a:pPr rtl="0"/>
@@ -6909,6 +6911,8 @@
   <cols>
     <col min="1" max="1" width="23.6640625" customWidth="1"/>
     <col min="2" max="2" width="22.53125" customWidth="1"/>
+    <col min="11" max="11" width="18.46484375" customWidth="1"/>
+    <col min="12" max="12" width="20.53125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.45">

</xml_diff>